<commit_message>
Result6: drop degenerate hybrid H_bm5_cos5; best F1 back to M1 (0.426)
A "hybrid" whose cosine-k equals the BM25 prefilter (BM25->5 then cosine->5)
returns exactly the BM25 top-k set -- the rerank is a no-op -- so it is not a
hybrid at all. H_bm5_cos5 was such a config and was misleadingly the top scorer.

Removed the run and regenerated the derived artifacts (summary.json,
master_summary, best_per_category, Excel). With it gone the best method is
M1 (markdown top-2 cosine, F1 0.426); best genuine hybrids are the k=8 runs
(H_bm15_cos8 0.417, H_bm10_cos8 0.413). SUMMARY.md updated to explain and
reflect this.

Signed-off-by: Daniel Nguyen <danielnguyenh07@gmail.com>
</commit_message>
<xml_diff>
--- a/RAG_Research/Result6/evaluation_by_category.xlsx
+++ b/RAG_Research/Result6/evaluation_by_category.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="128">
   <si>
     <t>method</t>
   </si>
@@ -275,6 +275,9 @@
     <t>hybrid</t>
   </si>
   <si>
+    <t>H_bm5_cos3</t>
+  </si>
+  <si>
     <t>R@k = of gold reachable in that method's chunks, fraction whose chunk is in the top-k retrieved. reach = coverage*R@k. X|R = of retrieved gold, fraction the LLM then extracted. M3 bypasses retrieval (full-contract check).</t>
   </si>
   <si>
@@ -326,7 +329,7 @@
     <t>best method (Jaccard)</t>
   </si>
   <si>
-    <t>H_bm5_cos5</t>
+    <t>H_bm10_cos1</t>
   </si>
   <si>
     <t>M2_top1_cosine</t>
@@ -336,9 +339,6 @@
   </si>
   <si>
     <t>M7_section_hybrid_top5</t>
-  </si>
-  <si>
-    <t>H_bm10_cos1</t>
   </si>
   <si>
     <t>H_bm15_cos2</t>
@@ -372,9 +372,6 @@
   </si>
   <si>
     <t>H_bm10_cos2</t>
-  </si>
-  <si>
-    <t>H_bm5_cos3</t>
   </si>
   <si>
     <t>How many categories each method wins (best F1):</t>
@@ -3835,9 +3832,9 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>Recall_at_k!$A$2:$A$8</c:f>
+              <c:f>Recall_at_k!$A$2:$A$9</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>M1 md top2-cos</c:v>
                 </c:pt>
@@ -3858,16 +3855,19 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>M7 sec hybrid-5</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>H_bm5_cos3</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Recall_at_k!$F$2:$F$8</c:f>
+              <c:f>Recall_at_k!$F$2:$F$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>0.9330000000000001</c:v>
                 </c:pt>
@@ -3887,6 +3887,9 @@
                   <c:v>0.989</c:v>
                 </c:pt>
                 <c:pt idx="6">
+                  <c:v>0.989</c:v>
+                </c:pt>
+                <c:pt idx="7">
                   <c:v>0.989</c:v>
                 </c:pt>
               </c:numCache>
@@ -3901,9 +3904,9 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>Recall_at_k!$A$2:$A$8</c:f>
+              <c:f>Recall_at_k!$A$2:$A$9</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>M1 md top2-cos</c:v>
                 </c:pt>
@@ -3924,16 +3927,19 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>M7 sec hybrid-5</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>H_bm5_cos3</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Recall_at_k!$G$2:$G$8</c:f>
+              <c:f>Recall_at_k!$G$2:$G$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>0.623</c:v>
                 </c:pt>
@@ -3954,6 +3960,9 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0.655</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.588</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3967,9 +3976,9 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>Recall_at_k!$A$2:$A$8</c:f>
+              <c:f>Recall_at_k!$A$2:$A$9</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>M1 md top2-cos</c:v>
                 </c:pt>
@@ -3990,16 +3999,19 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>M7 sec hybrid-5</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>H_bm5_cos3</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Recall_at_k!$H$2:$H$8</c:f>
+              <c:f>Recall_at_k!$H$2:$H$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>0.581</c:v>
                 </c:pt>
@@ -4020,6 +4032,9 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0.648</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.581</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4033,9 +4048,9 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>Recall_at_k!$A$2:$A$8</c:f>
+              <c:f>Recall_at_k!$A$2:$A$9</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>M1 md top2-cos</c:v>
                 </c:pt>
@@ -4056,16 +4071,19 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>M7 sec hybrid-5</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>H_bm5_cos3</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Recall_at_k!$I$2:$I$8</c:f>
+              <c:f>Recall_at_k!$I$2:$I$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>0.712</c:v>
                 </c:pt>
@@ -4086,6 +4104,9 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0.647</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.644</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4099,9 +4120,9 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>Recall_at_k!$A$2:$A$8</c:f>
+              <c:f>Recall_at_k!$A$2:$A$9</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>M1 md top2-cos</c:v>
                 </c:pt>
@@ -4122,16 +4143,19 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>M7 sec hybrid-5</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>H_bm5_cos3</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Recall_at_k!$J$2:$J$8</c:f>
+              <c:f>Recall_at_k!$J$2:$J$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>0.436</c:v>
                 </c:pt>
@@ -4152,6 +4176,9 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0.425</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.391</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4308,13 +4335,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>12</xdr:row>
+      <xdr:row>13</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
       <xdr:colOff>314325</xdr:colOff>
-      <xdr:row>40</xdr:row>
+      <xdr:row>41</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -13451,7 +13478,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30.7109375" customWidth="1"/>
@@ -13714,9 +13741,41 @@
         <v>0.425</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
-      <c r="A10" s="2" t="s">
+    <row r="9" spans="1:10">
+      <c r="A9" s="2" t="s">
         <v>84</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D9" s="3">
+        <v>3</v>
+      </c>
+      <c r="E9" s="3">
+        <v>220</v>
+      </c>
+      <c r="F9" s="4">
+        <v>0.989</v>
+      </c>
+      <c r="G9" s="4">
+        <v>0.588</v>
+      </c>
+      <c r="H9" s="4">
+        <v>0.581</v>
+      </c>
+      <c r="I9" s="4">
+        <v>0.644</v>
+      </c>
+      <c r="J9" s="4">
+        <v>0.391</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -13736,12 +13795,12 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>6</v>
@@ -13753,18 +13812,18 @@
         <v>5</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>75</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B3" s="4">
         <v>0.3123</v>
@@ -13787,7 +13846,7 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B4" s="4">
         <v>0.3813</v>
@@ -13810,7 +13869,7 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B5" s="4">
         <v>0.4011</v>
@@ -13833,58 +13892,34 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="B6" s="4">
-        <v>0.4304</v>
-      </c>
-      <c r="C6" s="4">
-        <v>0.4059</v>
-      </c>
-      <c r="D6" s="4">
-        <v>0.4581</v>
-      </c>
-      <c r="E6" s="4">
-        <v>0.5266</v>
-      </c>
-      <c r="F6" s="4">
-        <v>0.6384</v>
-      </c>
-      <c r="G6" s="4">
-        <v>0.577377</v>
-      </c>
+        <v>93</v>
+      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="B7" s="4">
-        <v>0.4304</v>
-      </c>
-      <c r="C7" s="4">
-        <v>0.4059</v>
-      </c>
-      <c r="D7" s="4">
-        <v>0.4581</v>
-      </c>
-      <c r="E7" s="4">
-        <v>0.5266</v>
-      </c>
-      <c r="F7" s="4">
-        <v>0.6384</v>
-      </c>
-      <c r="G7" s="4">
-        <v>0.577377</v>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>6</v>
@@ -13896,18 +13931,18 @@
         <v>5</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>75</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B12" s="4">
         <v>0.2707</v>
@@ -13930,7 +13965,7 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B13" s="4">
         <v>0.3666</v>
@@ -13953,7 +13988,7 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B14" s="4">
         <v>0.3953</v>
@@ -13976,7 +14011,7 @@
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B15" s="4">
         <v>0.3938</v>
@@ -13999,7 +14034,7 @@
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B16" s="4">
         <v>0.4131</v>
@@ -14022,12 +14057,12 @@
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>6</v>
@@ -14039,18 +14074,18 @@
         <v>5</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>75</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B21" s="4">
         <v>0.2711</v>
@@ -14073,7 +14108,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B22" s="4">
         <v>0.3387</v>
@@ -14096,7 +14131,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B23" s="4">
         <v>0.3837</v>
@@ -14119,7 +14154,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B24" s="4">
         <v>0.4011</v>
@@ -14142,7 +14177,7 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B25" s="4">
         <v>0.4167</v>
@@ -14165,7 +14200,7 @@
     </row>
     <row r="28" spans="1:7">
       <c r="A28" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -14187,16 +14222,16 @@
         <v>21</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>26</v>
@@ -14210,16 +14245,16 @@
         <v>8</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D2" s="4">
         <v>0</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F2" s="4">
-        <v>0.0717</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -14230,13 +14265,13 @@
         <v>6</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D3" s="4">
         <v>0.25</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F3" s="4">
         <v>0.3833</v>
@@ -14250,13 +14285,13 @@
         <v>6</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D4" s="4">
         <v>0.25</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F4" s="4">
         <v>0.7601</v>
@@ -14270,7 +14305,7 @@
         <v>5</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D5" s="4">
         <v>0.2857</v>
@@ -14336,7 +14371,7 @@
         <v>0.4</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F8" s="4">
         <v>0.6528</v>
@@ -14376,7 +14411,7 @@
         <v>0.4286</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F10" s="4">
         <v>0.4973</v>
@@ -14390,13 +14425,13 @@
         <v>6</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D11" s="4">
         <v>0.4444</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F11" s="4">
         <v>0.4744</v>
@@ -14410,13 +14445,13 @@
         <v>3</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D12" s="4">
         <v>0.5</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F12" s="4">
         <v>0.6435</v>
@@ -14450,13 +14485,13 @@
         <v>3</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D14" s="4">
         <v>0.5714</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F14" s="4">
         <v>0.6714</v>
@@ -14496,7 +14531,7 @@
         <v>0.5881999999999999</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F16" s="4">
         <v>0.5161</v>
@@ -14516,7 +14551,7 @@
         <v>0.6</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F17" s="4">
         <v>0.4911</v>
@@ -14530,13 +14565,13 @@
         <v>5</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D18" s="4">
         <v>0.6667</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F18" s="4">
         <v>0.6686</v>
@@ -14576,7 +14611,7 @@
         <v>0.6667</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="F20" s="4">
         <v>0.875</v>
@@ -14610,13 +14645,13 @@
         <v>5</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>101</v>
+        <v>84</v>
       </c>
       <c r="D22" s="4">
-        <v>0.8</v>
+        <v>0.75</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F22" s="4">
         <v>0.7947</v>
@@ -14730,13 +14765,13 @@
         <v>1</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D28" s="4">
         <v>1</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F28" s="4">
         <v>0.5881999999999999</v>
@@ -14816,7 +14851,7 @@
         <v>1</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>117</v>
+        <v>84</v>
       </c>
       <c r="F32" s="4">
         <v>0.9787</v>
@@ -14824,7 +14859,7 @@
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -14853,7 +14888,7 @@
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B38" s="3">
         <v>3</v>
@@ -14864,12 +14899,12 @@
         <v>102</v>
       </c>
       <c r="B39" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="2" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="B40" s="3">
         <v>2</v>
@@ -14877,7 +14912,7 @@
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="2" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="B41" s="3">
         <v>2</v>
@@ -14885,15 +14920,15 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" s="2" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="B42" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B43" s="3">
         <v>1</v>
@@ -14901,7 +14936,7 @@
     </row>
     <row r="44" spans="1:2">
       <c r="A44" s="2" t="s">
-        <v>110</v>
+        <v>84</v>
       </c>
       <c r="B44" s="3">
         <v>1</v>
@@ -14941,7 +14976,7 @@
     </row>
     <row r="49" spans="1:2">
       <c r="A49" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B49" s="3">
         <v>1</v>
@@ -14954,7 +14989,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T20"/>
+  <dimension ref="A1:T19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="26.7109375" customWidth="1"/>
@@ -14966,7 +15001,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>71</v>
@@ -14975,7 +15010,7 @@
         <v>72</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>73</v>
@@ -14996,22 +15031,22 @@
         <v>8</v>
       </c>
       <c r="L1" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>125</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>126</v>
       </c>
       <c r="R1" s="1" t="s">
         <v>74</v>
@@ -15020,7 +15055,7 @@
         <v>75</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:20">
@@ -15085,7 +15120,7 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>79</v>
@@ -15387,7 +15422,7 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>82</v>
@@ -15449,7 +15484,7 @@
     </row>
     <row r="9" spans="1:20">
       <c r="A9" s="2" t="s">
-        <v>117</v>
+        <v>84</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>82</v>
@@ -15511,7 +15546,7 @@
     </row>
     <row r="10" spans="1:20">
       <c r="A10" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>82</v>
@@ -15520,60 +15555,60 @@
         <v>83</v>
       </c>
       <c r="D10" s="3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E10" s="2">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F10" s="3">
         <v>220</v>
       </c>
       <c r="G10" s="4">
-        <v>0.4304</v>
+        <v>0.2707</v>
       </c>
       <c r="H10" s="4">
-        <v>0.4059</v>
+        <v>0.4138</v>
       </c>
       <c r="I10" s="4">
-        <v>0.4581</v>
+        <v>0.2011</v>
       </c>
       <c r="J10" s="4">
-        <v>0.4466</v>
+        <v>0.2242</v>
       </c>
       <c r="K10" s="4">
-        <v>0.322</v>
+        <v>0.1422</v>
       </c>
       <c r="L10" s="4">
-        <v>0.4304</v>
+        <v>0.2707</v>
       </c>
       <c r="M10" s="4">
-        <v>0.5266</v>
+        <v>0.2599</v>
       </c>
       <c r="N10" s="4">
-        <v>1</v>
+        <v>0.9902</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="P10" s="4">
         <v>0</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="R10" s="4">
         <v>0.9888</v>
       </c>
       <c r="S10" s="4">
-        <v>0.6384</v>
+        <v>0.2881</v>
       </c>
       <c r="T10" s="4">
-        <v>0.577377</v>
+        <v>0.208193</v>
       </c>
     </row>
     <row r="11" spans="1:20">
       <c r="A11" s="2" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>82</v>
@@ -15582,7 +15617,7 @@
         <v>83</v>
       </c>
       <c r="D11" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E11" s="2">
         <v>10</v>
@@ -15591,31 +15626,31 @@
         <v>220</v>
       </c>
       <c r="G11" s="4">
-        <v>0.2707</v>
+        <v>0.3666</v>
       </c>
       <c r="H11" s="4">
-        <v>0.4138</v>
+        <v>0.4318</v>
       </c>
       <c r="I11" s="4">
-        <v>0.2011</v>
+        <v>0.3184</v>
       </c>
       <c r="J11" s="4">
-        <v>0.2242</v>
+        <v>0.3361</v>
       </c>
       <c r="K11" s="4">
-        <v>0.1422</v>
+        <v>0.228</v>
       </c>
       <c r="L11" s="4">
-        <v>0.2707</v>
+        <v>0.3666</v>
       </c>
       <c r="M11" s="4">
-        <v>0.2599</v>
+        <v>0.3743</v>
       </c>
       <c r="N11" s="4">
-        <v>0.9902</v>
+        <v>1</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="P11" s="4">
         <v>0</v>
@@ -15627,15 +15662,15 @@
         <v>0.9888</v>
       </c>
       <c r="S11" s="4">
-        <v>0.2881</v>
+        <v>0.4407</v>
       </c>
       <c r="T11" s="4">
-        <v>0.208193</v>
+        <v>0.309878</v>
       </c>
     </row>
     <row r="12" spans="1:20">
       <c r="A12" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>82</v>
@@ -15644,7 +15679,7 @@
         <v>83</v>
       </c>
       <c r="D12" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12" s="2">
         <v>10</v>
@@ -15653,31 +15688,31 @@
         <v>220</v>
       </c>
       <c r="G12" s="4">
-        <v>0.3666</v>
+        <v>0.3953</v>
       </c>
       <c r="H12" s="4">
-        <v>0.4318</v>
+        <v>0.4121</v>
       </c>
       <c r="I12" s="4">
-        <v>0.3184</v>
+        <v>0.3799</v>
       </c>
       <c r="J12" s="4">
-        <v>0.3361</v>
+        <v>0.3859</v>
       </c>
       <c r="K12" s="4">
-        <v>0.228</v>
+        <v>0.2682</v>
       </c>
       <c r="L12" s="4">
-        <v>0.3666</v>
+        <v>0.3953</v>
       </c>
       <c r="M12" s="4">
-        <v>0.3743</v>
+        <v>0.39</v>
       </c>
       <c r="N12" s="4">
         <v>1</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="P12" s="4">
         <v>0</v>
@@ -15689,15 +15724,15 @@
         <v>0.9888</v>
       </c>
       <c r="S12" s="4">
-        <v>0.4407</v>
+        <v>0.548</v>
       </c>
       <c r="T12" s="4">
-        <v>0.309878</v>
+        <v>0.407834</v>
       </c>
     </row>
     <row r="13" spans="1:20">
       <c r="A13" s="2" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>82</v>
@@ -15706,7 +15741,7 @@
         <v>83</v>
       </c>
       <c r="D13" s="3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E13" s="2">
         <v>10</v>
@@ -15715,25 +15750,25 @@
         <v>220</v>
       </c>
       <c r="G13" s="4">
-        <v>0.3953</v>
+        <v>0.3938</v>
       </c>
       <c r="H13" s="4">
-        <v>0.4121</v>
+        <v>0.3671</v>
       </c>
       <c r="I13" s="4">
-        <v>0.3799</v>
+        <v>0.4246</v>
       </c>
       <c r="J13" s="4">
-        <v>0.3859</v>
+        <v>0.4117</v>
       </c>
       <c r="K13" s="4">
-        <v>0.2682</v>
+        <v>0.2902</v>
       </c>
       <c r="L13" s="4">
-        <v>0.3953</v>
+        <v>0.3938</v>
       </c>
       <c r="M13" s="4">
-        <v>0.39</v>
+        <v>0.4801</v>
       </c>
       <c r="N13" s="4">
         <v>1</v>
@@ -15745,16 +15780,16 @@
         <v>0</v>
       </c>
       <c r="Q13" s="2" t="s">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="R13" s="4">
         <v>0.9888</v>
       </c>
       <c r="S13" s="4">
-        <v>0.548</v>
+        <v>0.6554</v>
       </c>
       <c r="T13" s="4">
-        <v>0.407834</v>
+        <v>0.575844</v>
       </c>
     </row>
     <row r="14" spans="1:20">
@@ -15768,7 +15803,7 @@
         <v>83</v>
       </c>
       <c r="D14" s="3">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E14" s="2">
         <v>10</v>
@@ -15777,31 +15812,31 @@
         <v>220</v>
       </c>
       <c r="G14" s="4">
-        <v>0.3938</v>
+        <v>0.4131</v>
       </c>
       <c r="H14" s="4">
-        <v>0.3671</v>
+        <v>0.3563</v>
       </c>
       <c r="I14" s="4">
-        <v>0.4246</v>
+        <v>0.4916</v>
       </c>
       <c r="J14" s="4">
-        <v>0.4117</v>
+        <v>0.4569</v>
       </c>
       <c r="K14" s="4">
-        <v>0.2902</v>
+        <v>0.3334</v>
       </c>
       <c r="L14" s="4">
-        <v>0.3938</v>
+        <v>0.4131</v>
       </c>
       <c r="M14" s="4">
-        <v>0.4801</v>
+        <v>0.5495</v>
       </c>
       <c r="N14" s="4">
         <v>1</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="P14" s="4">
         <v>0</v>
@@ -15813,15 +15848,15 @@
         <v>0.9888</v>
       </c>
       <c r="S14" s="4">
-        <v>0.6554</v>
+        <v>0.7458</v>
       </c>
       <c r="T14" s="4">
-        <v>0.575844</v>
+        <v>0.836446</v>
       </c>
     </row>
     <row r="15" spans="1:20">
       <c r="A15" s="2" t="s">
-        <v>103</v>
+        <v>127</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>82</v>
@@ -15830,60 +15865,60 @@
         <v>83</v>
       </c>
       <c r="D15" s="3">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E15" s="2">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F15" s="3">
         <v>220</v>
       </c>
       <c r="G15" s="4">
-        <v>0.4131</v>
+        <v>0.2711</v>
       </c>
       <c r="H15" s="4">
-        <v>0.3563</v>
+        <v>0.3936</v>
       </c>
       <c r="I15" s="4">
-        <v>0.4916</v>
+        <v>0.2067</v>
       </c>
       <c r="J15" s="4">
-        <v>0.4569</v>
+        <v>0.2284</v>
       </c>
       <c r="K15" s="4">
-        <v>0.3334</v>
+        <v>0.144</v>
       </c>
       <c r="L15" s="4">
-        <v>0.4131</v>
+        <v>0.2711</v>
       </c>
       <c r="M15" s="4">
-        <v>0.5495</v>
+        <v>0.286</v>
       </c>
       <c r="N15" s="4">
-        <v>1</v>
+        <v>0.9902</v>
       </c>
       <c r="O15" s="2" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="P15" s="4">
         <v>0</v>
       </c>
       <c r="Q15" s="2" t="s">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="R15" s="4">
         <v>0.9888</v>
       </c>
       <c r="S15" s="4">
-        <v>0.7458</v>
+        <v>0.3051</v>
       </c>
       <c r="T15" s="4">
-        <v>0.836446</v>
+        <v>0.208956</v>
       </c>
     </row>
     <row r="16" spans="1:20">
       <c r="A16" s="2" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>82</v>
@@ -15892,7 +15927,7 @@
         <v>83</v>
       </c>
       <c r="D16" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E16" s="2">
         <v>15</v>
@@ -15901,31 +15936,31 @@
         <v>220</v>
       </c>
       <c r="G16" s="4">
-        <v>0.2711</v>
+        <v>0.3387</v>
       </c>
       <c r="H16" s="4">
-        <v>0.3936</v>
+        <v>0.3955</v>
       </c>
       <c r="I16" s="4">
-        <v>0.2067</v>
+        <v>0.2961</v>
       </c>
       <c r="J16" s="4">
-        <v>0.2284</v>
+        <v>0.3118</v>
       </c>
       <c r="K16" s="4">
-        <v>0.144</v>
+        <v>0.2066</v>
       </c>
       <c r="L16" s="4">
-        <v>0.2711</v>
+        <v>0.3387</v>
       </c>
       <c r="M16" s="4">
-        <v>0.286</v>
+        <v>0.3267</v>
       </c>
       <c r="N16" s="4">
-        <v>0.9902</v>
+        <v>1</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="P16" s="4">
         <v>0</v>
@@ -15937,15 +15972,15 @@
         <v>0.9888</v>
       </c>
       <c r="S16" s="4">
-        <v>0.3051</v>
+        <v>0.4124</v>
       </c>
       <c r="T16" s="4">
-        <v>0.208956</v>
+        <v>0.308169</v>
       </c>
     </row>
     <row r="17" spans="1:20">
       <c r="A17" s="2" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>82</v>
@@ -15954,7 +15989,7 @@
         <v>83</v>
       </c>
       <c r="D17" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E17" s="2">
         <v>15</v>
@@ -15963,25 +15998,25 @@
         <v>220</v>
       </c>
       <c r="G17" s="4">
-        <v>0.3387</v>
+        <v>0.3837</v>
       </c>
       <c r="H17" s="4">
-        <v>0.3955</v>
+        <v>0.4</v>
       </c>
       <c r="I17" s="4">
-        <v>0.2961</v>
+        <v>0.3687</v>
       </c>
       <c r="J17" s="4">
-        <v>0.3118</v>
+        <v>0.3746</v>
       </c>
       <c r="K17" s="4">
-        <v>0.2066</v>
+        <v>0.2581</v>
       </c>
       <c r="L17" s="4">
-        <v>0.3387</v>
+        <v>0.3837</v>
       </c>
       <c r="M17" s="4">
-        <v>0.3267</v>
+        <v>0.3839</v>
       </c>
       <c r="N17" s="4">
         <v>1</v>
@@ -15999,15 +16034,15 @@
         <v>0.9888</v>
       </c>
       <c r="S17" s="4">
-        <v>0.4124</v>
+        <v>0.5254</v>
       </c>
       <c r="T17" s="4">
-        <v>0.308169</v>
+        <v>0.407829</v>
       </c>
     </row>
     <row r="18" spans="1:20">
       <c r="A18" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>82</v>
@@ -16016,7 +16051,7 @@
         <v>83</v>
       </c>
       <c r="D18" s="3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E18" s="2">
         <v>15</v>
@@ -16025,25 +16060,25 @@
         <v>220</v>
       </c>
       <c r="G18" s="4">
-        <v>0.3837</v>
+        <v>0.4011</v>
       </c>
       <c r="H18" s="4">
-        <v>0.4</v>
+        <v>0.38</v>
       </c>
       <c r="I18" s="4">
-        <v>0.3687</v>
+        <v>0.4246</v>
       </c>
       <c r="J18" s="4">
-        <v>0.3746</v>
+        <v>0.4148</v>
       </c>
       <c r="K18" s="4">
-        <v>0.2581</v>
+        <v>0.293</v>
       </c>
       <c r="L18" s="4">
-        <v>0.3837</v>
+        <v>0.4011</v>
       </c>
       <c r="M18" s="4">
-        <v>0.3839</v>
+        <v>0.4579</v>
       </c>
       <c r="N18" s="4">
         <v>1</v>
@@ -16055,21 +16090,21 @@
         <v>0</v>
       </c>
       <c r="Q18" s="2" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="R18" s="4">
         <v>0.9888</v>
       </c>
       <c r="S18" s="4">
-        <v>0.5254</v>
+        <v>0.6497000000000001</v>
       </c>
       <c r="T18" s="4">
-        <v>0.407829</v>
+        <v>0.574396</v>
       </c>
     </row>
     <row r="19" spans="1:20">
       <c r="A19" s="2" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>82</v>
@@ -16078,7 +16113,7 @@
         <v>83</v>
       </c>
       <c r="D19" s="3">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E19" s="2">
         <v>15</v>
@@ -16087,107 +16122,45 @@
         <v>220</v>
       </c>
       <c r="G19" s="4">
-        <v>0.4011</v>
+        <v>0.4167</v>
       </c>
       <c r="H19" s="4">
-        <v>0.38</v>
+        <v>0.3557</v>
       </c>
       <c r="I19" s="4">
-        <v>0.4246</v>
+        <v>0.5028</v>
       </c>
       <c r="J19" s="4">
-        <v>0.4148</v>
+        <v>0.4644</v>
       </c>
       <c r="K19" s="4">
-        <v>0.293</v>
+        <v>0.3408</v>
       </c>
       <c r="L19" s="4">
-        <v>0.4011</v>
+        <v>0.4167</v>
       </c>
       <c r="M19" s="4">
-        <v>0.4579</v>
+        <v>0.5393</v>
       </c>
       <c r="N19" s="4">
         <v>1</v>
       </c>
       <c r="O19" s="2" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="P19" s="4">
         <v>0</v>
       </c>
       <c r="Q19" s="2" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="R19" s="4">
         <v>0.9888</v>
       </c>
       <c r="S19" s="4">
-        <v>0.6497000000000001</v>
+        <v>0.7571</v>
       </c>
       <c r="T19" s="4">
-        <v>0.574396</v>
-      </c>
-    </row>
-    <row r="20" spans="1:20">
-      <c r="A20" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D20" s="3">
-        <v>8</v>
-      </c>
-      <c r="E20" s="2">
-        <v>15</v>
-      </c>
-      <c r="F20" s="3">
-        <v>220</v>
-      </c>
-      <c r="G20" s="4">
-        <v>0.4167</v>
-      </c>
-      <c r="H20" s="4">
-        <v>0.3557</v>
-      </c>
-      <c r="I20" s="4">
-        <v>0.5028</v>
-      </c>
-      <c r="J20" s="4">
-        <v>0.4644</v>
-      </c>
-      <c r="K20" s="4">
-        <v>0.3408</v>
-      </c>
-      <c r="L20" s="4">
-        <v>0.4167</v>
-      </c>
-      <c r="M20" s="4">
-        <v>0.5393</v>
-      </c>
-      <c r="N20" s="4">
-        <v>1</v>
-      </c>
-      <c r="O20" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P20" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="R20" s="4">
-        <v>0.9888</v>
-      </c>
-      <c r="S20" s="4">
-        <v>0.7571</v>
-      </c>
-      <c r="T20" s="4">
         <v>0.836769</v>
       </c>
     </row>

</xml_diff>